<commit_message>
financial model v2: add Unit Economics, 24-month projection, funding/returns, worst-case scenario
</commit_message>
<xml_diff>
--- a/marketing/WinWin-Financial-Model.xlsx
+++ b/marketing/WinWin-Financial-Model.xlsx
@@ -11,6 +11,9 @@
     <sheet name="النموذج" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="التحليل" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="الحساسية" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="الاقتصاد الوحدوي" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="التوقعات الشهرية" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="التمويل والعائد" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -19,13 +22,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);-"/>
     <numFmt numFmtId="165" formatCode="0.0%;(0.0%);-"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0x"/>
+    <numFmt numFmtId="168" formatCode="#,##0;(#,##0)"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -99,6 +103,17 @@
       <color rgb="00777777"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000E2254"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -154,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" readingOrder="2"/>
@@ -244,6 +259,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
     <xf numFmtId="167" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -257,6 +275,33 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -369,6 +414,26 @@
     <comment ref="B11" authorId="0" shapeId="0">
       <text>
         <t>التراكمي يتحول موجباً خلال السنة 4: 3 سنوات + (400,000 ÷ 1,800,000)</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>WINوWIN</author>
+  </authors>
+  <commentList>
+    <comment ref="B6" authorId="0" shapeId="0">
+      <text>
+        <t>نمو عضوي + إحالة → تكلفة منخفضة</t>
+      </text>
+    </comment>
+    <comment ref="C6" authorId="0" shapeId="0">
+      <text>
+        <t>جهد مبيعات مباشر</t>
       </text>
     </comment>
   </commentList>
@@ -1580,13 +1645,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1624,6 +1690,11 @@
           <t>متفائل</t>
         </is>
       </c>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>أسوأ حالة</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1631,14 +1702,17 @@
           <t>معامل النمو</t>
         </is>
       </c>
-      <c r="B5" s="31" t="n">
+      <c r="B5" s="32" t="n">
         <v>0.7</v>
       </c>
-      <c r="C5" s="31" t="n">
+      <c r="C5" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="31" t="n">
+      <c r="D5" s="32" t="n">
         <v>1.3</v>
+      </c>
+      <c r="E5" s="32" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="6">
@@ -1659,6 +1733,10 @@
         <f>الفرضيات!$B$7</f>
         <v/>
       </c>
+      <c r="E6" s="8">
+        <f>الفرضيات!$B$7</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1678,6 +1756,10 @@
         <f>D6*(1+الفرضيات!$B$8*D$5)</f>
         <v/>
       </c>
+      <c r="E7" s="8">
+        <f>E6*(1+الفرضيات!$B$8*E$5)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1697,6 +1779,10 @@
         <f>D7*(1+الفرضيات!$B$9*D$5)</f>
         <v/>
       </c>
+      <c r="E8" s="8">
+        <f>E7*(1+الفرضيات!$B$9*E$5)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1716,6 +1802,10 @@
         <f>D8*(1+الفرضيات!$B$10*D$5)</f>
         <v/>
       </c>
+      <c r="E9" s="8">
+        <f>E8*(1+الفرضيات!$B$10*E$5)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1735,6 +1825,10 @@
         <f>D9*(1+الفرضيات!$B$11*D$5)</f>
         <v/>
       </c>
+      <c r="E10" s="8">
+        <f>E9*(1+الفرضيات!$B$11*E$5)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1742,16 +1836,20 @@
           <t>الإيراد — السنة 1</t>
         </is>
       </c>
-      <c r="B12" s="32">
+      <c r="B12" s="33">
         <f>B6*الفرضيات!$B$17</f>
         <v/>
       </c>
-      <c r="C12" s="32">
+      <c r="C12" s="33">
         <f>C6*الفرضيات!$B$17</f>
         <v/>
       </c>
-      <c r="D12" s="32">
+      <c r="D12" s="33">
         <f>D6*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="E12" s="33">
+        <f>E6*الفرضيات!$B$17</f>
         <v/>
       </c>
     </row>
@@ -1761,16 +1859,20 @@
           <t>الإيراد — السنة 2</t>
         </is>
       </c>
-      <c r="B13" s="32">
+      <c r="B13" s="33">
         <f>B7*الفرضيات!$B$17</f>
         <v/>
       </c>
-      <c r="C13" s="32">
+      <c r="C13" s="33">
         <f>C7*الفرضيات!$B$17</f>
         <v/>
       </c>
-      <c r="D13" s="32">
+      <c r="D13" s="33">
         <f>D7*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="E13" s="33">
+        <f>E7*الفرضيات!$B$17</f>
         <v/>
       </c>
     </row>
@@ -1780,16 +1882,20 @@
           <t>الإيراد — السنة 3</t>
         </is>
       </c>
-      <c r="B14" s="32">
+      <c r="B14" s="33">
         <f>B8*الفرضيات!$B$17</f>
         <v/>
       </c>
-      <c r="C14" s="32">
+      <c r="C14" s="33">
         <f>C8*الفرضيات!$B$17</f>
         <v/>
       </c>
-      <c r="D14" s="32">
+      <c r="D14" s="33">
         <f>D8*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="E14" s="33">
+        <f>E8*الفرضيات!$B$17</f>
         <v/>
       </c>
     </row>
@@ -1799,16 +1905,20 @@
           <t>الإيراد — السنة 4</t>
         </is>
       </c>
-      <c r="B15" s="32">
+      <c r="B15" s="33">
         <f>B9*الفرضيات!$B$17</f>
         <v/>
       </c>
-      <c r="C15" s="32">
+      <c r="C15" s="33">
         <f>C9*الفرضيات!$B$17</f>
         <v/>
       </c>
-      <c r="D15" s="32">
+      <c r="D15" s="33">
         <f>D9*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="E15" s="33">
+        <f>E9*الفرضيات!$B$17</f>
         <v/>
       </c>
     </row>
@@ -1818,16 +1928,20 @@
           <t>الإيراد — السنة 5</t>
         </is>
       </c>
-      <c r="B16" s="32">
+      <c r="B16" s="33">
         <f>B10*الفرضيات!$B$17</f>
         <v/>
       </c>
-      <c r="C16" s="32">
+      <c r="C16" s="33">
         <f>C10*الفرضيات!$B$17</f>
         <v/>
       </c>
-      <c r="D16" s="32">
+      <c r="D16" s="33">
         <f>D10*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="E16" s="33">
+        <f>E10*الفرضيات!$B$17</f>
         <v/>
       </c>
     </row>
@@ -1849,6 +1963,10 @@
         <f>D12-الفرضيات!$B$30</f>
         <v/>
       </c>
+      <c r="E18" s="24">
+        <f>E12-الفرضيات!$B$30</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1868,6 +1986,10 @@
         <f>D13-الفرضيات!$C$30</f>
         <v/>
       </c>
+      <c r="E19" s="24">
+        <f>E13-الفرضيات!$C$30</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1887,6 +2009,10 @@
         <f>D14-الفرضيات!$D$30</f>
         <v/>
       </c>
+      <c r="E20" s="24">
+        <f>E14-الفرضيات!$D$30</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1906,6 +2032,10 @@
         <f>D15-الفرضيات!$E$30</f>
         <v/>
       </c>
+      <c r="E21" s="24">
+        <f>E15-الفرضيات!$E$30</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1925,6 +2055,10 @@
         <f>D16-الفرضيات!$F$30</f>
         <v/>
       </c>
+      <c r="E22" s="24">
+        <f>E16-الفرضيات!$F$30</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="20" t="inlineStr">
@@ -1932,16 +2066,20 @@
           <t>NPV @ معدل الخصم</t>
         </is>
       </c>
-      <c r="B24" s="33">
+      <c r="B24" s="34">
         <f>-الفرضيات!$B$21+NPV(الفرضيات!$B$22,0,0,B20,B21,B22)</f>
         <v/>
       </c>
-      <c r="C24" s="33">
+      <c r="C24" s="34">
         <f>-الفرضيات!$B$21+NPV(الفرضيات!$B$22,0,0,C20,C21,C22)</f>
         <v/>
       </c>
-      <c r="D24" s="33">
+      <c r="D24" s="34">
         <f>-الفرضيات!$B$21+NPV(الفرضيات!$B$22,0,0,D20,D21,D22)</f>
+        <v/>
+      </c>
+      <c r="E24" s="34">
+        <f>-الفرضيات!$B$21+NPV(الفرضيات!$B$22,0,0,E20,E21,E22)</f>
         <v/>
       </c>
     </row>
@@ -1951,16 +2089,20 @@
           <t>معدل العائد الداخلي IRR</t>
         </is>
       </c>
-      <c r="B25" s="34">
+      <c r="B25" s="35">
         <f>IFERROR(IRR(B28:B33),"غير محقق")</f>
         <v/>
       </c>
-      <c r="C25" s="34">
+      <c r="C25" s="35">
         <f>IFERROR(IRR(C28:C33),"غير محقق")</f>
         <v/>
       </c>
-      <c r="D25" s="34">
+      <c r="D25" s="35">
         <f>IFERROR(IRR(D28:D33),"غير محقق")</f>
+        <v/>
+      </c>
+      <c r="E25" s="35">
+        <f>IFERROR(IRR(E28:E33),"غير محقق")</f>
         <v/>
       </c>
     </row>
@@ -1977,15 +2119,19 @@
           <t>السنة 0</t>
         </is>
       </c>
-      <c r="B28" s="35">
+      <c r="B28" s="36">
         <f>-الفرضيات!$B$21</f>
         <v/>
       </c>
-      <c r="C28" s="35">
+      <c r="C28" s="36">
         <f>-الفرضيات!$B$21</f>
         <v/>
       </c>
-      <c r="D28" s="35">
+      <c r="D28" s="36">
+        <f>-الفرضيات!$B$21</f>
+        <v/>
+      </c>
+      <c r="E28" s="36">
         <f>-الفرضيات!$B$21</f>
         <v/>
       </c>
@@ -1996,13 +2142,16 @@
           <t>السنة 1</t>
         </is>
       </c>
-      <c r="B29" s="35" t="n">
+      <c r="B29" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="C29" s="35" t="n">
+      <c r="C29" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="D29" s="35" t="n">
+      <c r="D29" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2012,13 +2161,16 @@
           <t>السنة 2</t>
         </is>
       </c>
-      <c r="B30" s="35" t="n">
+      <c r="B30" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="C30" s="35" t="n">
+      <c r="C30" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="D30" s="35" t="n">
+      <c r="D30" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2028,16 +2180,20 @@
           <t>السنة 3</t>
         </is>
       </c>
-      <c r="B31" s="35">
+      <c r="B31" s="36">
         <f>B20</f>
         <v/>
       </c>
-      <c r="C31" s="35">
+      <c r="C31" s="36">
         <f>C20</f>
         <v/>
       </c>
-      <c r="D31" s="35">
+      <c r="D31" s="36">
         <f>D20</f>
+        <v/>
+      </c>
+      <c r="E31" s="36">
+        <f>E20</f>
         <v/>
       </c>
     </row>
@@ -2047,16 +2203,20 @@
           <t>السنة 4</t>
         </is>
       </c>
-      <c r="B32" s="35">
+      <c r="B32" s="36">
         <f>B21</f>
         <v/>
       </c>
-      <c r="C32" s="35">
+      <c r="C32" s="36">
         <f>C21</f>
         <v/>
       </c>
-      <c r="D32" s="35">
+      <c r="D32" s="36">
         <f>D21</f>
+        <v/>
+      </c>
+      <c r="E32" s="36">
+        <f>E21</f>
         <v/>
       </c>
     </row>
@@ -2066,17 +2226,1237 @@
           <t>السنة 5</t>
         </is>
       </c>
-      <c r="B33" s="35">
+      <c r="B33" s="36">
         <f>B22</f>
         <v/>
       </c>
-      <c r="C33" s="35">
+      <c r="C33" s="36">
         <f>C22</f>
         <v/>
       </c>
-      <c r="D33" s="35">
+      <c r="D33" s="36">
         <f>D22</f>
         <v/>
+      </c>
+      <c r="E33" s="36">
+        <f>E22</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>الاقتصاد الوحدوي (Unit Economics)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>يوضّح ربحية اكتساب كل مستخدم وكل براند — أساس قابلية التوسّع</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>المؤشر</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>المستخدم</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>البراند</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>عدد الوحدات — السنة 1</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>20000</v>
+      </c>
+      <c r="C5" s="37">
+        <f>الفرضيات!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>تكلفة الاكتساب CAC (ريال)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>إيراد المنصة لكل وحدة سنوياً (ريال)</t>
+        </is>
+      </c>
+      <c r="B7" s="33">
+        <f>النموذج!B5/B5</f>
+        <v/>
+      </c>
+      <c r="C7" s="33">
+        <f>الفرضيات!B6*الفرضيات!B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>متوسط بقاء الوحدة (سنوات)</t>
+        </is>
+      </c>
+      <c r="B8" s="38" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C8" s="38" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>هامش المساهمة</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>القيمة الدائمة LTV (ريال)</t>
+        </is>
+      </c>
+      <c r="B10" s="39">
+        <f>B7*B8*B9</f>
+        <v/>
+      </c>
+      <c r="C10" s="39">
+        <f>C7*C8*C9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>نسبة LTV/CAC</t>
+        </is>
+      </c>
+      <c r="B11" s="40">
+        <f>B10/B6</f>
+        <v/>
+      </c>
+      <c r="C11" s="40">
+        <f>C10/C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>قاعدة إبهام: LTV/CAC ≥ 3x تعني اكتساباً صحياً وقابلاً للتوسّع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>البراندات هي محرّك الربح الأساسي؛ المستخدمون يُكتسبون بتكلفة منخفضة لتغذية الشبكة.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>التوقعات الشهرية — أول 24 شهراً</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>مبنية على منحنى تصاعدي يوازي إجمالي السنة؛ الرصيد الافتتاحي = الاستثمار − التأسيس</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>الرصيد النقدي الافتتاحي</t>
+        </is>
+      </c>
+      <c r="B3" s="42">
+        <f>الفرضيات!B21-الفرضيات!B20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>الشهر</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>GMV</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>الإيراد</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>المصاريف</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>الصافي</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>الرصيد النقدي</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="43" t="inlineStr">
+        <is>
+          <t>شهر 1</t>
+        </is>
+      </c>
+      <c r="B6" s="8">
+        <f>النموذج!$B$4*(1/78)</f>
+        <v/>
+      </c>
+      <c r="C6" s="33">
+        <f>B6*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D6" s="8">
+        <f>الفرضيات!$B$30/12</f>
+        <v/>
+      </c>
+      <c r="E6" s="24">
+        <f>C6-D6</f>
+        <v/>
+      </c>
+      <c r="F6" s="26">
+        <f>B3+E6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="43" t="inlineStr">
+        <is>
+          <t>شهر 2</t>
+        </is>
+      </c>
+      <c r="B7" s="8">
+        <f>النموذج!$B$4*(2/78)</f>
+        <v/>
+      </c>
+      <c r="C7" s="33">
+        <f>B7*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D7" s="8">
+        <f>الفرضيات!$B$30/12</f>
+        <v/>
+      </c>
+      <c r="E7" s="24">
+        <f>C7-D7</f>
+        <v/>
+      </c>
+      <c r="F7" s="26">
+        <f>F6+E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="43" t="inlineStr">
+        <is>
+          <t>شهر 3</t>
+        </is>
+      </c>
+      <c r="B8" s="8">
+        <f>النموذج!$B$4*(3/78)</f>
+        <v/>
+      </c>
+      <c r="C8" s="33">
+        <f>B8*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D8" s="8">
+        <f>الفرضيات!$B$30/12</f>
+        <v/>
+      </c>
+      <c r="E8" s="24">
+        <f>C8-D8</f>
+        <v/>
+      </c>
+      <c r="F8" s="26">
+        <f>F7+E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="43" t="inlineStr">
+        <is>
+          <t>شهر 4</t>
+        </is>
+      </c>
+      <c r="B9" s="8">
+        <f>النموذج!$B$4*(4/78)</f>
+        <v/>
+      </c>
+      <c r="C9" s="33">
+        <f>B9*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D9" s="8">
+        <f>الفرضيات!$B$30/12</f>
+        <v/>
+      </c>
+      <c r="E9" s="24">
+        <f>C9-D9</f>
+        <v/>
+      </c>
+      <c r="F9" s="26">
+        <f>F8+E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="43" t="inlineStr">
+        <is>
+          <t>شهر 5</t>
+        </is>
+      </c>
+      <c r="B10" s="8">
+        <f>النموذج!$B$4*(5/78)</f>
+        <v/>
+      </c>
+      <c r="C10" s="33">
+        <f>B10*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D10" s="8">
+        <f>الفرضيات!$B$30/12</f>
+        <v/>
+      </c>
+      <c r="E10" s="24">
+        <f>C10-D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="26">
+        <f>F9+E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="43" t="inlineStr">
+        <is>
+          <t>شهر 6</t>
+        </is>
+      </c>
+      <c r="B11" s="8">
+        <f>النموذج!$B$4*(6/78)</f>
+        <v/>
+      </c>
+      <c r="C11" s="33">
+        <f>B11*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D11" s="8">
+        <f>الفرضيات!$B$30/12</f>
+        <v/>
+      </c>
+      <c r="E11" s="24">
+        <f>C11-D11</f>
+        <v/>
+      </c>
+      <c r="F11" s="26">
+        <f>F10+E11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="43" t="inlineStr">
+        <is>
+          <t>شهر 7</t>
+        </is>
+      </c>
+      <c r="B12" s="8">
+        <f>النموذج!$B$4*(7/78)</f>
+        <v/>
+      </c>
+      <c r="C12" s="33">
+        <f>B12*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D12" s="8">
+        <f>الفرضيات!$B$30/12</f>
+        <v/>
+      </c>
+      <c r="E12" s="24">
+        <f>C12-D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="26">
+        <f>F11+E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="43" t="inlineStr">
+        <is>
+          <t>شهر 8</t>
+        </is>
+      </c>
+      <c r="B13" s="8">
+        <f>النموذج!$B$4*(8/78)</f>
+        <v/>
+      </c>
+      <c r="C13" s="33">
+        <f>B13*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D13" s="8">
+        <f>الفرضيات!$B$30/12</f>
+        <v/>
+      </c>
+      <c r="E13" s="24">
+        <f>C13-D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="26">
+        <f>F12+E13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="43" t="inlineStr">
+        <is>
+          <t>شهر 9</t>
+        </is>
+      </c>
+      <c r="B14" s="8">
+        <f>النموذج!$B$4*(9/78)</f>
+        <v/>
+      </c>
+      <c r="C14" s="33">
+        <f>B14*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D14" s="8">
+        <f>الفرضيات!$B$30/12</f>
+        <v/>
+      </c>
+      <c r="E14" s="24">
+        <f>C14-D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="26">
+        <f>F13+E14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="43" t="inlineStr">
+        <is>
+          <t>شهر 10</t>
+        </is>
+      </c>
+      <c r="B15" s="8">
+        <f>النموذج!$B$4*(10/78)</f>
+        <v/>
+      </c>
+      <c r="C15" s="33">
+        <f>B15*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D15" s="8">
+        <f>الفرضيات!$B$30/12</f>
+        <v/>
+      </c>
+      <c r="E15" s="24">
+        <f>C15-D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="26">
+        <f>F14+E15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>شهر 11</t>
+        </is>
+      </c>
+      <c r="B16" s="8">
+        <f>النموذج!$B$4*(11/78)</f>
+        <v/>
+      </c>
+      <c r="C16" s="33">
+        <f>B16*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D16" s="8">
+        <f>الفرضيات!$B$30/12</f>
+        <v/>
+      </c>
+      <c r="E16" s="24">
+        <f>C16-D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="26">
+        <f>F15+E16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>شهر 12</t>
+        </is>
+      </c>
+      <c r="B17" s="8">
+        <f>النموذج!$B$4*(12/78)</f>
+        <v/>
+      </c>
+      <c r="C17" s="33">
+        <f>B17*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D17" s="8">
+        <f>الفرضيات!$B$30/12</f>
+        <v/>
+      </c>
+      <c r="E17" s="24">
+        <f>C17-D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="26">
+        <f>F16+E17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>شهر 13</t>
+        </is>
+      </c>
+      <c r="B18" s="8">
+        <f>النموذج!$C$4*(1/78)</f>
+        <v/>
+      </c>
+      <c r="C18" s="33">
+        <f>B18*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D18" s="8">
+        <f>الفرضيات!$C$30/12</f>
+        <v/>
+      </c>
+      <c r="E18" s="24">
+        <f>C18-D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="26">
+        <f>F17+E18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="43" t="inlineStr">
+        <is>
+          <t>شهر 14</t>
+        </is>
+      </c>
+      <c r="B19" s="8">
+        <f>النموذج!$C$4*(2/78)</f>
+        <v/>
+      </c>
+      <c r="C19" s="33">
+        <f>B19*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D19" s="8">
+        <f>الفرضيات!$C$30/12</f>
+        <v/>
+      </c>
+      <c r="E19" s="24">
+        <f>C19-D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="26">
+        <f>F18+E19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="43" t="inlineStr">
+        <is>
+          <t>شهر 15</t>
+        </is>
+      </c>
+      <c r="B20" s="8">
+        <f>النموذج!$C$4*(3/78)</f>
+        <v/>
+      </c>
+      <c r="C20" s="33">
+        <f>B20*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D20" s="8">
+        <f>الفرضيات!$C$30/12</f>
+        <v/>
+      </c>
+      <c r="E20" s="24">
+        <f>C20-D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="26">
+        <f>F19+E20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="43" t="inlineStr">
+        <is>
+          <t>شهر 16</t>
+        </is>
+      </c>
+      <c r="B21" s="8">
+        <f>النموذج!$C$4*(4/78)</f>
+        <v/>
+      </c>
+      <c r="C21" s="33">
+        <f>B21*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D21" s="8">
+        <f>الفرضيات!$C$30/12</f>
+        <v/>
+      </c>
+      <c r="E21" s="24">
+        <f>C21-D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="26">
+        <f>F20+E21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="43" t="inlineStr">
+        <is>
+          <t>شهر 17</t>
+        </is>
+      </c>
+      <c r="B22" s="8">
+        <f>النموذج!$C$4*(5/78)</f>
+        <v/>
+      </c>
+      <c r="C22" s="33">
+        <f>B22*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D22" s="8">
+        <f>الفرضيات!$C$30/12</f>
+        <v/>
+      </c>
+      <c r="E22" s="24">
+        <f>C22-D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="26">
+        <f>F21+E22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="43" t="inlineStr">
+        <is>
+          <t>شهر 18</t>
+        </is>
+      </c>
+      <c r="B23" s="8">
+        <f>النموذج!$C$4*(6/78)</f>
+        <v/>
+      </c>
+      <c r="C23" s="33">
+        <f>B23*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D23" s="8">
+        <f>الفرضيات!$C$30/12</f>
+        <v/>
+      </c>
+      <c r="E23" s="24">
+        <f>C23-D23</f>
+        <v/>
+      </c>
+      <c r="F23" s="26">
+        <f>F22+E23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="43" t="inlineStr">
+        <is>
+          <t>شهر 19</t>
+        </is>
+      </c>
+      <c r="B24" s="8">
+        <f>النموذج!$C$4*(7/78)</f>
+        <v/>
+      </c>
+      <c r="C24" s="33">
+        <f>B24*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D24" s="8">
+        <f>الفرضيات!$C$30/12</f>
+        <v/>
+      </c>
+      <c r="E24" s="24">
+        <f>C24-D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="26">
+        <f>F23+E24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="43" t="inlineStr">
+        <is>
+          <t>شهر 20</t>
+        </is>
+      </c>
+      <c r="B25" s="8">
+        <f>النموذج!$C$4*(8/78)</f>
+        <v/>
+      </c>
+      <c r="C25" s="33">
+        <f>B25*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D25" s="8">
+        <f>الفرضيات!$C$30/12</f>
+        <v/>
+      </c>
+      <c r="E25" s="24">
+        <f>C25-D25</f>
+        <v/>
+      </c>
+      <c r="F25" s="26">
+        <f>F24+E25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="43" t="inlineStr">
+        <is>
+          <t>شهر 21</t>
+        </is>
+      </c>
+      <c r="B26" s="8">
+        <f>النموذج!$C$4*(9/78)</f>
+        <v/>
+      </c>
+      <c r="C26" s="33">
+        <f>B26*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D26" s="8">
+        <f>الفرضيات!$C$30/12</f>
+        <v/>
+      </c>
+      <c r="E26" s="24">
+        <f>C26-D26</f>
+        <v/>
+      </c>
+      <c r="F26" s="26">
+        <f>F25+E26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="43" t="inlineStr">
+        <is>
+          <t>شهر 22</t>
+        </is>
+      </c>
+      <c r="B27" s="8">
+        <f>النموذج!$C$4*(10/78)</f>
+        <v/>
+      </c>
+      <c r="C27" s="33">
+        <f>B27*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D27" s="8">
+        <f>الفرضيات!$C$30/12</f>
+        <v/>
+      </c>
+      <c r="E27" s="24">
+        <f>C27-D27</f>
+        <v/>
+      </c>
+      <c r="F27" s="26">
+        <f>F26+E27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="43" t="inlineStr">
+        <is>
+          <t>شهر 23</t>
+        </is>
+      </c>
+      <c r="B28" s="8">
+        <f>النموذج!$C$4*(11/78)</f>
+        <v/>
+      </c>
+      <c r="C28" s="33">
+        <f>B28*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D28" s="8">
+        <f>الفرضيات!$C$30/12</f>
+        <v/>
+      </c>
+      <c r="E28" s="24">
+        <f>C28-D28</f>
+        <v/>
+      </c>
+      <c r="F28" s="26">
+        <f>F27+E28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="43" t="inlineStr">
+        <is>
+          <t>شهر 24</t>
+        </is>
+      </c>
+      <c r="B29" s="8">
+        <f>النموذج!$C$4*(12/78)</f>
+        <v/>
+      </c>
+      <c r="C29" s="33">
+        <f>B29*الفرضيات!$B$17</f>
+        <v/>
+      </c>
+      <c r="D29" s="8">
+        <f>الفرضيات!$C$30/12</f>
+        <v/>
+      </c>
+      <c r="E29" s="24">
+        <f>C29-D29</f>
+        <v/>
+      </c>
+      <c r="F29" s="26">
+        <f>F28+E29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>أدنى رصيد نقدي خلال 24 شهراً</t>
+        </is>
+      </c>
+      <c r="B31" s="26">
+        <f>MIN(F6:F29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>متوسط الحرق الشهري — السنة 1 (Burn)</t>
+        </is>
+      </c>
+      <c r="B32" s="44">
+        <f>AVERAGE(E6:E17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>الرصيد النقدي بنهاية الشهر 24</t>
+        </is>
+      </c>
+      <c r="B33" s="26">
+        <f>F29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>ملاحظة: بقاء أدنى رصيد موجباً = كفاية الاستثمار حتى الوصول للربحية.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>خطة استخدام التمويل والعائد للمستثمر</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>أرقام التقييم والعائد استرشادية وقابلة للتفاوض</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>أولاً: استخدام التمويل (1.2 مليون ريال)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>البند</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>النسبة</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>المبلغ (ريال)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>التسويق والنمو</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C6" s="8">
+        <f>B6*الفرضيات!$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>الرواتب والفريق</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C7" s="8">
+        <f>B7*الفرضيات!$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>التقنية والبنية والـ SMS</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C8" s="8">
+        <f>B8*الفرضيات!$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>قانوني وتراخيص وإداري</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C9" s="8">
+        <f>B9*الفرضيات!$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>احتياطي نقدي</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C10" s="8">
+        <f>B10*الفرضيات!$B$21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="B11" s="45">
+        <f>SUM(B6:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="21">
+        <f>SUM(C6:C10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>ثانياً: شروط الاستثمار (استرشادي)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>مبلغ الجولة</t>
+        </is>
+      </c>
+      <c r="B14" s="19">
+        <f>الفرضيات!B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>حصة المستثمر</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>التقييم بعد الجولة (Post-money)</t>
+        </is>
+      </c>
+      <c r="B16" s="26">
+        <f>B14/B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>التقييم قبل الجولة (Pre-money)</t>
+        </is>
+      </c>
+      <c r="B17" s="26">
+        <f>B16-B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>حصة المؤسسين</t>
+        </is>
+      </c>
+      <c r="B18" s="29">
+        <f>1-B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>ثالثاً: تقدير العائد عند الخروج (السنة 5)</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>مضاعف التقييم على الإيراد (Revenue Multiple)</t>
+        </is>
+      </c>
+      <c r="B21" s="32" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>إيراد السنة 5</t>
+        </is>
+      </c>
+      <c r="B22" s="19">
+        <f>النموذج!F5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>قيمة الشركة عند الخروج</t>
+        </is>
+      </c>
+      <c r="B23" s="26">
+        <f>B21*B22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>حصة المستثمر عند الخروج</t>
+        </is>
+      </c>
+      <c r="B24" s="26">
+        <f>B23*B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>مضاعف رأس المال MOIC</t>
+        </is>
+      </c>
+      <c r="B25" s="40">
+        <f>B24/B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>معدل العائد السنوي التقريبي على 5 سنوات</t>
+        </is>
+      </c>
+      <c r="B26" s="27">
+        <f>(B24/B14)^(1/5)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>خطة الخروج: استحواذ استراتيجي (مجموعات إعلام/تسويق أو منصة إقليمية)، أو بيع حصص، أو إدراج مستقبلي في السوق الموازية (نمو). الأفق 5–7 سنوات.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>